<commit_message>
20250813-1529 Get 202507 salemon data.
</commit_message>
<xml_diff>
--- a/Data/EXCEL/Transfer/salemon/202507-1/1101-salemon-202507.xlsx
+++ b/Data/EXCEL/Transfer/salemon/202507-1/1101-salemon-202507.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WORKSPACES\xls2xlsx\Transfer\202507\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{466EBD44-F0F2-4876-9C17-44B1A89F9A52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2A58DEB9-D825-4FAA-ABA8-EB121D20ADAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6180" yWindow="585" windowWidth="21750" windowHeight="13170" xr2:uid="{0580B8BB-F4ED-4F63-9FD9-723FA4C083D0}"/>
+    <workbookView xWindow="6525" yWindow="930" windowWidth="21750" windowHeight="13170" xr2:uid="{259ABB33-A539-4964-AF33-1F1E907CAF4B}"/>
   </bookViews>
   <sheets>
     <sheet name="1101-salemon-202507" sheetId="2" r:id="rId1"/>
@@ -863,10 +863,10 @@
     <xf numFmtId="0" fontId="23" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="22" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="3" fontId="22" fillId="33" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="22" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1261,8 +1261,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB130041-AD3D-49E2-A014-395001A374AF}">
-  <dimension ref="A1:Q43"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A93BA7BE-09F1-46F9-A2C7-E121F655A5B5}">
+  <dimension ref="A1:Q44"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.875" customWidth="1"/>
@@ -1429,2068 +1429,2121 @@
     </row>
     <row r="5" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
-        <v>45809</v>
+        <v>45839</v>
       </c>
       <c r="B5" s="6">
-        <v>29.05</v>
+        <v>25.8</v>
       </c>
       <c r="C5" s="6">
-        <v>25.5</v>
+        <v>24.3</v>
       </c>
       <c r="D5" s="6">
-        <v>29.05</v>
+        <v>26.6</v>
       </c>
       <c r="E5" s="6">
-        <v>24.75</v>
+        <v>22.9</v>
       </c>
       <c r="F5" s="7">
-        <v>-3.85</v>
+        <v>-1.2</v>
       </c>
       <c r="G5" s="7">
-        <v>-13.12</v>
+        <v>-4.71</v>
       </c>
       <c r="H5" s="8">
-        <v>101.1</v>
-      </c>
-      <c r="I5" s="7">
-        <v>-19.899999999999999</v>
+        <v>135.4</v>
+      </c>
+      <c r="I5" s="9">
+        <v>33.9</v>
       </c>
       <c r="J5" s="7">
-        <v>-26</v>
+        <v>-6.19</v>
       </c>
       <c r="K5" s="8">
-        <v>703.8</v>
+        <v>839.2</v>
       </c>
       <c r="L5" s="9">
-        <v>8.5500000000000007</v>
+        <v>5.87</v>
       </c>
       <c r="M5" s="8">
-        <v>101.1</v>
-      </c>
-      <c r="N5" s="7">
-        <v>-19.899999999999999</v>
+        <v>135.4</v>
+      </c>
+      <c r="N5" s="9">
+        <v>33.9</v>
       </c>
       <c r="O5" s="7">
-        <v>-26</v>
+        <v>-6.19</v>
       </c>
       <c r="P5" s="8">
-        <v>703.8</v>
+        <v>839.2</v>
       </c>
       <c r="Q5" s="9">
-        <v>8.5500000000000007</v>
+        <v>5.87</v>
       </c>
     </row>
     <row r="6" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11">
-        <v>45778</v>
+        <v>45809</v>
       </c>
       <c r="B6" s="12">
-        <v>29.9</v>
+        <v>29.05</v>
       </c>
       <c r="C6" s="12">
-        <v>29.35</v>
+        <v>25.5</v>
       </c>
       <c r="D6" s="12">
-        <v>31.4</v>
+        <v>29.05</v>
       </c>
       <c r="E6" s="12">
-        <v>28.7</v>
+        <v>24.75</v>
       </c>
       <c r="F6" s="13">
-        <v>-0.3</v>
+        <v>-3.85</v>
       </c>
       <c r="G6" s="13">
-        <v>-1.01</v>
+        <v>-13.12</v>
       </c>
       <c r="H6" s="14">
-        <v>126.2</v>
+        <v>101.1</v>
       </c>
       <c r="I6" s="13">
-        <v>-0.48</v>
+        <v>-19.899999999999999</v>
       </c>
       <c r="J6" s="13">
-        <v>-8.9499999999999993</v>
+        <v>-26</v>
       </c>
       <c r="K6" s="14">
-        <v>602.70000000000005</v>
+        <v>703.8</v>
       </c>
       <c r="L6" s="15">
-        <v>17.8</v>
+        <v>8.5500000000000007</v>
       </c>
       <c r="M6" s="14">
-        <v>126.2</v>
+        <v>101.1</v>
       </c>
       <c r="N6" s="13">
-        <v>-0.48</v>
+        <v>-19.899999999999999</v>
       </c>
       <c r="O6" s="13">
-        <v>-8.9499999999999993</v>
+        <v>-26</v>
       </c>
       <c r="P6" s="14">
-        <v>602.70000000000005</v>
+        <v>703.8</v>
       </c>
       <c r="Q6" s="15">
-        <v>17.8</v>
+        <v>8.5500000000000007</v>
       </c>
     </row>
     <row r="7" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
-        <v>45748</v>
+        <v>45778</v>
       </c>
       <c r="B7" s="6">
-        <v>32.15</v>
+        <v>29.9</v>
       </c>
       <c r="C7" s="6">
-        <v>29.65</v>
+        <v>29.35</v>
       </c>
       <c r="D7" s="6">
-        <v>32.65</v>
+        <v>31.4</v>
       </c>
       <c r="E7" s="6">
-        <v>28.45</v>
+        <v>28.7</v>
       </c>
       <c r="F7" s="7">
-        <v>-2.4</v>
+        <v>-0.3</v>
       </c>
       <c r="G7" s="7">
-        <v>-7.49</v>
+        <v>-1.01</v>
       </c>
       <c r="H7" s="8">
-        <v>126.8</v>
+        <v>126.2</v>
       </c>
       <c r="I7" s="7">
-        <v>-6.99</v>
-      </c>
-      <c r="J7" s="9">
-        <v>9.07</v>
+        <v>-0.48</v>
+      </c>
+      <c r="J7" s="7">
+        <v>-8.9499999999999993</v>
       </c>
       <c r="K7" s="8">
-        <v>476.5</v>
+        <v>602.70000000000005</v>
       </c>
       <c r="L7" s="9">
-        <v>27.7</v>
+        <v>17.8</v>
       </c>
       <c r="M7" s="8">
-        <v>126.8</v>
+        <v>126.2</v>
       </c>
       <c r="N7" s="7">
-        <v>-6.99</v>
-      </c>
-      <c r="O7" s="9">
-        <v>9.07</v>
+        <v>-0.48</v>
+      </c>
+      <c r="O7" s="7">
+        <v>-8.9499999999999993</v>
       </c>
       <c r="P7" s="8">
-        <v>476.5</v>
+        <v>602.70000000000005</v>
       </c>
       <c r="Q7" s="9">
-        <v>27.7</v>
+        <v>17.8</v>
       </c>
     </row>
     <row r="8" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11">
-        <v>45717</v>
+        <v>45748</v>
       </c>
       <c r="B8" s="12">
-        <v>34.4</v>
+        <v>32.15</v>
       </c>
       <c r="C8" s="12">
-        <v>32.049999999999997</v>
+        <v>29.65</v>
       </c>
       <c r="D8" s="12">
-        <v>35.450000000000003</v>
+        <v>32.65</v>
       </c>
       <c r="E8" s="12">
-        <v>32</v>
+        <v>28.45</v>
       </c>
       <c r="F8" s="13">
-        <v>-3.05</v>
+        <v>-2.4</v>
       </c>
       <c r="G8" s="13">
-        <v>-8.69</v>
+        <v>-7.49</v>
       </c>
       <c r="H8" s="14">
-        <v>136.4</v>
-      </c>
-      <c r="I8" s="15">
-        <v>49.4</v>
-      </c>
-      <c r="J8" s="13">
-        <v>-0.1</v>
+        <v>126.8</v>
+      </c>
+      <c r="I8" s="13">
+        <v>-6.99</v>
+      </c>
+      <c r="J8" s="15">
+        <v>9.07</v>
       </c>
       <c r="K8" s="14">
-        <v>349.7</v>
+        <v>476.5</v>
       </c>
       <c r="L8" s="15">
-        <v>36.200000000000003</v>
+        <v>27.7</v>
       </c>
       <c r="M8" s="14">
-        <v>136.4</v>
-      </c>
-      <c r="N8" s="15">
-        <v>49.4</v>
-      </c>
-      <c r="O8" s="13">
-        <v>-0.1</v>
+        <v>126.8</v>
+      </c>
+      <c r="N8" s="13">
+        <v>-6.99</v>
+      </c>
+      <c r="O8" s="15">
+        <v>9.07</v>
       </c>
       <c r="P8" s="14">
-        <v>349.7</v>
+        <v>476.5</v>
       </c>
       <c r="Q8" s="15">
-        <v>36.200000000000003</v>
+        <v>27.7</v>
       </c>
     </row>
     <row r="9" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
-        <v>45689</v>
+        <v>45717</v>
       </c>
       <c r="B9" s="6">
-        <v>31.55</v>
+        <v>34.4</v>
       </c>
       <c r="C9" s="6">
-        <v>35.1</v>
+        <v>32.049999999999997</v>
       </c>
       <c r="D9" s="6">
-        <v>35.35</v>
+        <v>35.450000000000003</v>
       </c>
       <c r="E9" s="6">
-        <v>30.85</v>
-      </c>
-      <c r="F9" s="9">
-        <v>3.25</v>
-      </c>
-      <c r="G9" s="9">
-        <v>10.199999999999999</v>
+        <v>32</v>
+      </c>
+      <c r="F9" s="7">
+        <v>-3.05</v>
+      </c>
+      <c r="G9" s="7">
+        <v>-8.69</v>
       </c>
       <c r="H9" s="8">
-        <v>91.23</v>
-      </c>
-      <c r="I9" s="7">
-        <v>-25.3</v>
-      </c>
-      <c r="J9" s="9">
-        <v>90.1</v>
+        <v>136.4</v>
+      </c>
+      <c r="I9" s="9">
+        <v>49.4</v>
+      </c>
+      <c r="J9" s="7">
+        <v>-0.1</v>
       </c>
       <c r="K9" s="8">
-        <v>213.4</v>
+        <v>349.7</v>
       </c>
       <c r="L9" s="9">
-        <v>77.3</v>
+        <v>36.200000000000003</v>
       </c>
       <c r="M9" s="8">
-        <v>91.23</v>
-      </c>
-      <c r="N9" s="7">
-        <v>-25.3</v>
-      </c>
-      <c r="O9" s="9">
-        <v>90.1</v>
+        <v>136.4</v>
+      </c>
+      <c r="N9" s="9">
+        <v>49.4</v>
+      </c>
+      <c r="O9" s="7">
+        <v>-0.1</v>
       </c>
       <c r="P9" s="8">
-        <v>213.4</v>
+        <v>349.7</v>
       </c>
       <c r="Q9" s="9">
-        <v>77.3</v>
+        <v>36.200000000000003</v>
       </c>
     </row>
     <row r="10" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11">
-        <v>45658</v>
+        <v>45689</v>
       </c>
       <c r="B10" s="12">
         <v>31.55</v>
       </c>
       <c r="C10" s="12">
-        <v>31.85</v>
+        <v>35.1</v>
       </c>
       <c r="D10" s="12">
-        <v>32</v>
+        <v>35.35</v>
       </c>
       <c r="E10" s="12">
-        <v>30.05</v>
+        <v>30.85</v>
       </c>
       <c r="F10" s="15">
-        <v>0.15</v>
+        <v>3.25</v>
       </c>
       <c r="G10" s="15">
-        <v>0.47</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="H10" s="14">
-        <v>122.1</v>
+        <v>91.23</v>
       </c>
       <c r="I10" s="13">
-        <v>-26.2</v>
+        <v>-25.3</v>
       </c>
       <c r="J10" s="15">
-        <v>68.7</v>
+        <v>90.1</v>
       </c>
       <c r="K10" s="14">
-        <v>122.1</v>
+        <v>213.4</v>
       </c>
       <c r="L10" s="15">
-        <v>68.7</v>
+        <v>77.3</v>
       </c>
       <c r="M10" s="14">
-        <v>122.1</v>
+        <v>91.23</v>
       </c>
       <c r="N10" s="13">
-        <v>-26.2</v>
+        <v>-25.3</v>
       </c>
       <c r="O10" s="15">
-        <v>68.7</v>
+        <v>90.1</v>
       </c>
       <c r="P10" s="14">
-        <v>122.1</v>
+        <v>213.4</v>
       </c>
       <c r="Q10" s="15">
-        <v>68.7</v>
+        <v>77.3</v>
       </c>
     </row>
     <row r="11" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
-        <v>45627</v>
+        <v>45658</v>
       </c>
       <c r="B11" s="6">
-        <v>33.6</v>
+        <v>31.55</v>
       </c>
       <c r="C11" s="6">
-        <v>31.7</v>
+        <v>31.85</v>
       </c>
       <c r="D11" s="6">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E11" s="6">
-        <v>31.4</v>
-      </c>
-      <c r="F11" s="7">
-        <v>-1.8</v>
-      </c>
-      <c r="G11" s="7">
-        <v>-5.37</v>
+        <v>30.05</v>
+      </c>
+      <c r="F11" s="9">
+        <v>0.15</v>
+      </c>
+      <c r="G11" s="9">
+        <v>0.47</v>
       </c>
       <c r="H11" s="8">
-        <v>165.4</v>
-      </c>
-      <c r="I11" s="9">
-        <v>0.24</v>
+        <v>122.1</v>
+      </c>
+      <c r="I11" s="7">
+        <v>-26.2</v>
       </c>
       <c r="J11" s="9">
-        <v>73.900000000000006</v>
-      </c>
-      <c r="K11" s="16">
-        <v>1549</v>
+        <v>68.7</v>
+      </c>
+      <c r="K11" s="8">
+        <v>122.1</v>
       </c>
       <c r="L11" s="9">
-        <v>42.6</v>
+        <v>68.7</v>
       </c>
       <c r="M11" s="8">
-        <v>165.4</v>
-      </c>
-      <c r="N11" s="9">
-        <v>0.24</v>
+        <v>122.1</v>
+      </c>
+      <c r="N11" s="7">
+        <v>-26.2</v>
       </c>
       <c r="O11" s="9">
-        <v>73.900000000000006</v>
-      </c>
-      <c r="P11" s="16">
-        <v>1549</v>
+        <v>68.7</v>
+      </c>
+      <c r="P11" s="8">
+        <v>122.1</v>
       </c>
       <c r="Q11" s="9">
-        <v>42.6</v>
+        <v>68.7</v>
       </c>
     </row>
     <row r="12" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11">
-        <v>45597</v>
+        <v>45627</v>
       </c>
       <c r="B12" s="12">
+        <v>33.6</v>
+      </c>
+      <c r="C12" s="12">
         <v>31.7</v>
       </c>
-      <c r="C12" s="12">
-        <v>33.5</v>
-      </c>
       <c r="D12" s="12">
-        <v>34.200000000000003</v>
+        <v>34</v>
       </c>
       <c r="E12" s="12">
-        <v>31.7</v>
-      </c>
-      <c r="F12" s="15">
-        <v>1.55</v>
-      </c>
-      <c r="G12" s="15">
-        <v>4.8499999999999996</v>
+        <v>31.4</v>
+      </c>
+      <c r="F12" s="13">
+        <v>-1.8</v>
+      </c>
+      <c r="G12" s="13">
+        <v>-5.37</v>
       </c>
       <c r="H12" s="14">
-        <v>165</v>
+        <v>165.4</v>
       </c>
       <c r="I12" s="15">
-        <v>1.41</v>
+        <v>0.24</v>
       </c>
       <c r="J12" s="15">
-        <v>87.8</v>
-      </c>
-      <c r="K12" s="17">
-        <v>1384</v>
+        <v>73.900000000000006</v>
+      </c>
+      <c r="K12" s="16">
+        <v>1549</v>
       </c>
       <c r="L12" s="15">
-        <v>39.6</v>
+        <v>42.6</v>
       </c>
       <c r="M12" s="14">
-        <v>165</v>
+        <v>165.4</v>
       </c>
       <c r="N12" s="15">
-        <v>1.41</v>
+        <v>0.24</v>
       </c>
       <c r="O12" s="15">
-        <v>87.8</v>
-      </c>
-      <c r="P12" s="17">
-        <v>1384</v>
+        <v>73.900000000000006</v>
+      </c>
+      <c r="P12" s="16">
+        <v>1549</v>
       </c>
       <c r="Q12" s="15">
-        <v>39.6</v>
+        <v>42.6</v>
       </c>
     </row>
     <row r="13" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
-        <v>45566</v>
+        <v>45597</v>
       </c>
       <c r="B13" s="6">
-        <v>33.9</v>
+        <v>31.7</v>
       </c>
       <c r="C13" s="6">
-        <v>31.95</v>
+        <v>33.5</v>
       </c>
       <c r="D13" s="6">
-        <v>34</v>
+        <v>34.200000000000003</v>
       </c>
       <c r="E13" s="6">
-        <v>31.75</v>
-      </c>
-      <c r="F13" s="7">
-        <v>-1.85</v>
-      </c>
-      <c r="G13" s="7">
-        <v>-5.47</v>
+        <v>31.7</v>
+      </c>
+      <c r="F13" s="9">
+        <v>1.55</v>
+      </c>
+      <c r="G13" s="9">
+        <v>4.8499999999999996</v>
       </c>
       <c r="H13" s="8">
-        <v>162.69999999999999</v>
+        <v>165</v>
       </c>
       <c r="I13" s="9">
-        <v>22.1</v>
+        <v>1.41</v>
       </c>
       <c r="J13" s="9">
-        <v>73.599999999999994</v>
-      </c>
-      <c r="K13" s="16">
-        <v>1219</v>
+        <v>87.8</v>
+      </c>
+      <c r="K13" s="17">
+        <v>1384</v>
       </c>
       <c r="L13" s="9">
-        <v>34.9</v>
+        <v>39.6</v>
       </c>
       <c r="M13" s="8">
-        <v>162.69999999999999</v>
+        <v>165</v>
       </c>
       <c r="N13" s="9">
-        <v>22.1</v>
+        <v>1.41</v>
       </c>
       <c r="O13" s="9">
-        <v>73.599999999999994</v>
-      </c>
-      <c r="P13" s="16">
-        <v>1219</v>
+        <v>87.8</v>
+      </c>
+      <c r="P13" s="17">
+        <v>1384</v>
       </c>
       <c r="Q13" s="9">
-        <v>34.9</v>
+        <v>39.6</v>
       </c>
     </row>
     <row r="14" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="11">
-        <v>45536</v>
+        <v>45566</v>
       </c>
       <c r="B14" s="12">
-        <v>32.9</v>
+        <v>33.9</v>
       </c>
       <c r="C14" s="12">
-        <v>33.799999999999997</v>
+        <v>31.95</v>
       </c>
       <c r="D14" s="12">
-        <v>34.200000000000003</v>
+        <v>34</v>
       </c>
       <c r="E14" s="12">
-        <v>31.2</v>
-      </c>
-      <c r="F14" s="15">
-        <v>0.85</v>
-      </c>
-      <c r="G14" s="15">
-        <v>2.58</v>
+        <v>31.75</v>
+      </c>
+      <c r="F14" s="13">
+        <v>-1.85</v>
+      </c>
+      <c r="G14" s="13">
+        <v>-5.47</v>
       </c>
       <c r="H14" s="14">
-        <v>133.30000000000001</v>
+        <v>162.69999999999999</v>
       </c>
       <c r="I14" s="15">
-        <v>2.46</v>
+        <v>22.1</v>
       </c>
       <c r="J14" s="15">
-        <v>52.5</v>
-      </c>
-      <c r="K14" s="17">
-        <v>1056</v>
+        <v>73.599999999999994</v>
+      </c>
+      <c r="K14" s="16">
+        <v>1219</v>
       </c>
       <c r="L14" s="15">
-        <v>30.4</v>
+        <v>34.9</v>
       </c>
       <c r="M14" s="14">
-        <v>133.30000000000001</v>
+        <v>162.69999999999999</v>
       </c>
       <c r="N14" s="15">
-        <v>2.46</v>
+        <v>22.1</v>
       </c>
       <c r="O14" s="15">
-        <v>52.5</v>
-      </c>
-      <c r="P14" s="17">
-        <v>1056</v>
+        <v>73.599999999999994</v>
+      </c>
+      <c r="P14" s="16">
+        <v>1219</v>
       </c>
       <c r="Q14" s="15">
-        <v>30.4</v>
+        <v>34.9</v>
       </c>
     </row>
     <row r="15" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
-        <v>45505</v>
+        <v>45536</v>
       </c>
       <c r="B15" s="6">
-        <v>34.65</v>
+        <v>32.9</v>
       </c>
       <c r="C15" s="6">
-        <v>32.950000000000003</v>
+        <v>33.799999999999997</v>
       </c>
       <c r="D15" s="6">
-        <v>34.799999999999997</v>
+        <v>34.200000000000003</v>
       </c>
       <c r="E15" s="6">
-        <v>32.5</v>
-      </c>
-      <c r="F15" s="7">
-        <v>-1.7</v>
-      </c>
-      <c r="G15" s="7">
-        <v>-4.91</v>
+        <v>31.2</v>
+      </c>
+      <c r="F15" s="9">
+        <v>0.85</v>
+      </c>
+      <c r="G15" s="9">
+        <v>2.58</v>
       </c>
       <c r="H15" s="8">
-        <v>130</v>
-      </c>
-      <c r="I15" s="7">
-        <v>-9.8699999999999992</v>
+        <v>133.30000000000001</v>
+      </c>
+      <c r="I15" s="9">
+        <v>2.46</v>
       </c>
       <c r="J15" s="9">
-        <v>38.6</v>
-      </c>
-      <c r="K15" s="8">
-        <v>922.7</v>
+        <v>52.5</v>
+      </c>
+      <c r="K15" s="17">
+        <v>1056</v>
       </c>
       <c r="L15" s="9">
-        <v>27.8</v>
+        <v>30.4</v>
       </c>
       <c r="M15" s="8">
-        <v>130</v>
-      </c>
-      <c r="N15" s="7">
-        <v>-9.8699999999999992</v>
+        <v>133.30000000000001</v>
+      </c>
+      <c r="N15" s="9">
+        <v>2.46</v>
       </c>
       <c r="O15" s="9">
-        <v>38.6</v>
-      </c>
-      <c r="P15" s="8">
-        <v>922.7</v>
+        <v>52.5</v>
+      </c>
+      <c r="P15" s="17">
+        <v>1056</v>
       </c>
       <c r="Q15" s="9">
-        <v>27.8</v>
+        <v>30.4</v>
       </c>
     </row>
     <row r="16" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="11">
-        <v>45474</v>
+        <v>45505</v>
       </c>
       <c r="B16" s="12">
-        <v>33.6</v>
+        <v>34.65</v>
       </c>
       <c r="C16" s="12">
-        <v>34.65</v>
+        <v>32.950000000000003</v>
       </c>
       <c r="D16" s="12">
-        <v>35.200000000000003</v>
+        <v>34.799999999999997</v>
       </c>
       <c r="E16" s="12">
-        <v>33.4</v>
-      </c>
-      <c r="F16" s="15">
-        <v>0.45</v>
-      </c>
-      <c r="G16" s="15">
-        <v>1.32</v>
+        <v>32.5</v>
+      </c>
+      <c r="F16" s="13">
+        <v>-1.7</v>
+      </c>
+      <c r="G16" s="13">
+        <v>-4.91</v>
       </c>
       <c r="H16" s="14">
-        <v>144.30000000000001</v>
-      </c>
-      <c r="I16" s="15">
-        <v>5.63</v>
+        <v>130</v>
+      </c>
+      <c r="I16" s="13">
+        <v>-9.8699999999999992</v>
       </c>
       <c r="J16" s="15">
-        <v>61.2</v>
+        <v>38.6</v>
       </c>
       <c r="K16" s="14">
-        <v>792.6</v>
+        <v>922.7</v>
       </c>
       <c r="L16" s="15">
-        <v>26.2</v>
+        <v>27.8</v>
       </c>
       <c r="M16" s="14">
-        <v>144.30000000000001</v>
-      </c>
-      <c r="N16" s="15">
-        <v>5.63</v>
+        <v>130</v>
+      </c>
+      <c r="N16" s="13">
+        <v>-9.8699999999999992</v>
       </c>
       <c r="O16" s="15">
-        <v>61.2</v>
+        <v>38.6</v>
       </c>
       <c r="P16" s="14">
-        <v>792.6</v>
+        <v>922.7</v>
       </c>
       <c r="Q16" s="15">
-        <v>26.2</v>
+        <v>27.8</v>
       </c>
     </row>
     <row r="17" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
-        <v>45444</v>
+        <v>45474</v>
       </c>
       <c r="B17" s="6">
-        <v>33.1</v>
+        <v>33.6</v>
       </c>
       <c r="C17" s="6">
-        <v>34.200000000000003</v>
+        <v>34.65</v>
       </c>
       <c r="D17" s="6">
-        <v>34.75</v>
+        <v>35.200000000000003</v>
       </c>
       <c r="E17" s="6">
-        <v>32.65</v>
+        <v>33.4</v>
       </c>
       <c r="F17" s="9">
-        <v>1.2</v>
+        <v>0.45</v>
       </c>
       <c r="G17" s="9">
-        <v>3.64</v>
+        <v>1.32</v>
       </c>
       <c r="H17" s="8">
-        <v>136.6</v>
-      </c>
-      <c r="I17" s="7">
-        <v>-1.44</v>
+        <v>144.30000000000001</v>
+      </c>
+      <c r="I17" s="9">
+        <v>5.63</v>
       </c>
       <c r="J17" s="9">
-        <v>54.9</v>
+        <v>61.2</v>
       </c>
       <c r="K17" s="8">
-        <v>648.29999999999995</v>
+        <v>792.6</v>
       </c>
       <c r="L17" s="9">
-        <v>20.3</v>
+        <v>26.2</v>
       </c>
       <c r="M17" s="8">
-        <v>136.6</v>
-      </c>
-      <c r="N17" s="7">
-        <v>-1.44</v>
+        <v>144.30000000000001</v>
+      </c>
+      <c r="N17" s="9">
+        <v>5.63</v>
       </c>
       <c r="O17" s="9">
-        <v>54.9</v>
+        <v>61.2</v>
       </c>
       <c r="P17" s="8">
-        <v>648.29999999999995</v>
+        <v>792.6</v>
       </c>
       <c r="Q17" s="9">
-        <v>20.3</v>
+        <v>26.2</v>
       </c>
     </row>
     <row r="18" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>45413</v>
+        <v>45444</v>
       </c>
       <c r="B18" s="12">
-        <v>32.1</v>
+        <v>33.1</v>
       </c>
       <c r="C18" s="12">
-        <v>33</v>
+        <v>34.200000000000003</v>
       </c>
       <c r="D18" s="12">
-        <v>34.4</v>
+        <v>34.75</v>
       </c>
       <c r="E18" s="12">
-        <v>32.1</v>
+        <v>32.65</v>
       </c>
       <c r="F18" s="15">
-        <v>0.95</v>
+        <v>1.2</v>
       </c>
       <c r="G18" s="15">
-        <v>2.96</v>
+        <v>3.64</v>
       </c>
       <c r="H18" s="14">
-        <v>138.6</v>
-      </c>
-      <c r="I18" s="15">
-        <v>19.2</v>
+        <v>136.6</v>
+      </c>
+      <c r="I18" s="13">
+        <v>-1.44</v>
       </c>
       <c r="J18" s="15">
-        <v>44.4</v>
+        <v>54.9</v>
       </c>
       <c r="K18" s="14">
-        <v>511.7</v>
+        <v>648.29999999999995</v>
       </c>
       <c r="L18" s="15">
-        <v>13.6</v>
+        <v>20.3</v>
       </c>
       <c r="M18" s="14">
-        <v>138.6</v>
-      </c>
-      <c r="N18" s="15">
-        <v>19.2</v>
+        <v>136.6</v>
+      </c>
+      <c r="N18" s="13">
+        <v>-1.44</v>
       </c>
       <c r="O18" s="15">
-        <v>44.4</v>
+        <v>54.9</v>
       </c>
       <c r="P18" s="14">
-        <v>511.7</v>
+        <v>648.29999999999995</v>
       </c>
       <c r="Q18" s="15">
-        <v>13.6</v>
+        <v>20.3</v>
       </c>
     </row>
     <row r="19" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
-        <v>45383</v>
+        <v>45413</v>
       </c>
       <c r="B19" s="6">
-        <v>32.25</v>
+        <v>32.1</v>
       </c>
       <c r="C19" s="6">
-        <v>32.049999999999997</v>
+        <v>33</v>
       </c>
       <c r="D19" s="6">
-        <v>33.6</v>
+        <v>34.4</v>
       </c>
       <c r="E19" s="6">
-        <v>31.75</v>
-      </c>
-      <c r="F19" s="7">
-        <v>-0.1</v>
-      </c>
-      <c r="G19" s="7">
-        <v>-0.31</v>
+        <v>32.1</v>
+      </c>
+      <c r="F19" s="9">
+        <v>0.95</v>
+      </c>
+      <c r="G19" s="9">
+        <v>2.96</v>
       </c>
       <c r="H19" s="8">
-        <v>116.3</v>
-      </c>
-      <c r="I19" s="7">
-        <v>-14.8</v>
+        <v>138.6</v>
+      </c>
+      <c r="I19" s="9">
+        <v>19.2</v>
       </c>
       <c r="J19" s="9">
-        <v>27.8</v>
+        <v>44.4</v>
       </c>
       <c r="K19" s="8">
-        <v>373.1</v>
+        <v>511.7</v>
       </c>
       <c r="L19" s="9">
-        <v>5.21</v>
+        <v>13.6</v>
       </c>
       <c r="M19" s="8">
-        <v>116.3</v>
-      </c>
-      <c r="N19" s="7">
-        <v>-14.8</v>
+        <v>138.6</v>
+      </c>
+      <c r="N19" s="9">
+        <v>19.2</v>
       </c>
       <c r="O19" s="9">
-        <v>27.8</v>
+        <v>44.4</v>
       </c>
       <c r="P19" s="8">
-        <v>373.1</v>
+        <v>511.7</v>
       </c>
       <c r="Q19" s="9">
-        <v>5.21</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="20" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="11">
-        <v>45352</v>
+        <v>45383</v>
       </c>
       <c r="B20" s="12">
-        <v>32.15</v>
+        <v>32.25</v>
       </c>
       <c r="C20" s="12">
-        <v>32.15</v>
+        <v>32.049999999999997</v>
       </c>
       <c r="D20" s="12">
-        <v>32.299999999999997</v>
+        <v>33.6</v>
       </c>
       <c r="E20" s="12">
-        <v>30.8</v>
-      </c>
-      <c r="F20" s="15">
-        <v>0.05</v>
-      </c>
-      <c r="G20" s="15">
-        <v>0.16</v>
+        <v>31.75</v>
+      </c>
+      <c r="F20" s="13">
+        <v>-0.1</v>
+      </c>
+      <c r="G20" s="13">
+        <v>-0.31</v>
       </c>
       <c r="H20" s="14">
-        <v>136.5</v>
-      </c>
-      <c r="I20" s="15">
-        <v>184.4</v>
+        <v>116.3</v>
+      </c>
+      <c r="I20" s="13">
+        <v>-14.8</v>
       </c>
       <c r="J20" s="15">
-        <v>16.399999999999999</v>
+        <v>27.8</v>
       </c>
       <c r="K20" s="14">
-        <v>256.89999999999998</v>
-      </c>
-      <c r="L20" s="13">
-        <v>-2.56</v>
+        <v>373.1</v>
+      </c>
+      <c r="L20" s="15">
+        <v>5.21</v>
       </c>
       <c r="M20" s="14">
-        <v>136.5</v>
-      </c>
-      <c r="N20" s="15">
-        <v>184.4</v>
+        <v>116.3</v>
+      </c>
+      <c r="N20" s="13">
+        <v>-14.8</v>
       </c>
       <c r="O20" s="15">
-        <v>16.399999999999999</v>
+        <v>27.8</v>
       </c>
       <c r="P20" s="14">
-        <v>256.89999999999998</v>
-      </c>
-      <c r="Q20" s="13">
-        <v>-2.56</v>
+        <v>373.1</v>
+      </c>
+      <c r="Q20" s="15">
+        <v>5.21</v>
       </c>
     </row>
     <row r="21" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
-        <v>45323</v>
+        <v>45352</v>
       </c>
       <c r="B21" s="6">
-        <v>31.95</v>
+        <v>32.15</v>
       </c>
       <c r="C21" s="6">
-        <v>32.1</v>
+        <v>32.15</v>
       </c>
       <c r="D21" s="6">
-        <v>32.9</v>
+        <v>32.299999999999997</v>
       </c>
       <c r="E21" s="6">
-        <v>31.8</v>
+        <v>30.8</v>
       </c>
       <c r="F21" s="9">
-        <v>0.2</v>
+        <v>0.05</v>
       </c>
       <c r="G21" s="9">
-        <v>0.63</v>
+        <v>0.16</v>
       </c>
       <c r="H21" s="8">
-        <v>47.99</v>
-      </c>
-      <c r="I21" s="7">
-        <v>-33.700000000000003</v>
-      </c>
-      <c r="J21" s="7">
-        <v>-34.299999999999997</v>
+        <v>136.5</v>
+      </c>
+      <c r="I21" s="9">
+        <v>184.4</v>
+      </c>
+      <c r="J21" s="9">
+        <v>16.399999999999999</v>
       </c>
       <c r="K21" s="8">
-        <v>120.4</v>
+        <v>256.89999999999998</v>
       </c>
       <c r="L21" s="7">
-        <v>-17.7</v>
+        <v>-2.56</v>
       </c>
       <c r="M21" s="8">
-        <v>47.99</v>
-      </c>
-      <c r="N21" s="7">
-        <v>-33.700000000000003</v>
-      </c>
-      <c r="O21" s="7">
-        <v>-34.299999999999997</v>
+        <v>136.5</v>
+      </c>
+      <c r="N21" s="9">
+        <v>184.4</v>
+      </c>
+      <c r="O21" s="9">
+        <v>16.399999999999999</v>
       </c>
       <c r="P21" s="8">
-        <v>120.4</v>
+        <v>256.89999999999998</v>
       </c>
       <c r="Q21" s="7">
-        <v>-17.7</v>
+        <v>-2.56</v>
       </c>
     </row>
     <row r="22" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="11">
-        <v>45292</v>
+        <v>45323</v>
       </c>
       <c r="B22" s="12">
-        <v>34.85</v>
+        <v>31.95</v>
       </c>
       <c r="C22" s="12">
-        <v>31.9</v>
+        <v>32.1</v>
       </c>
       <c r="D22" s="12">
-        <v>34.85</v>
+        <v>32.9</v>
       </c>
       <c r="E22" s="12">
         <v>31.8</v>
       </c>
-      <c r="F22" s="13">
-        <v>-2.95</v>
-      </c>
-      <c r="G22" s="13">
-        <v>-8.4600000000000009</v>
+      <c r="F22" s="15">
+        <v>0.2</v>
+      </c>
+      <c r="G22" s="15">
+        <v>0.63</v>
       </c>
       <c r="H22" s="14">
-        <v>72.38</v>
+        <v>47.99</v>
       </c>
       <c r="I22" s="13">
-        <v>-23.9</v>
+        <v>-33.700000000000003</v>
       </c>
       <c r="J22" s="13">
-        <v>-1.19</v>
+        <v>-34.299999999999997</v>
       </c>
       <c r="K22" s="14">
-        <v>72.38</v>
+        <v>120.4</v>
       </c>
       <c r="L22" s="13">
-        <v>-1.19</v>
+        <v>-17.7</v>
       </c>
       <c r="M22" s="14">
-        <v>72.38</v>
+        <v>47.99</v>
       </c>
       <c r="N22" s="13">
-        <v>-23.9</v>
+        <v>-33.700000000000003</v>
       </c>
       <c r="O22" s="13">
-        <v>-1.19</v>
+        <v>-34.299999999999997</v>
       </c>
       <c r="P22" s="14">
-        <v>72.38</v>
+        <v>120.4</v>
       </c>
       <c r="Q22" s="13">
-        <v>-1.19</v>
+        <v>-17.7</v>
       </c>
     </row>
     <row r="23" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
-        <v>45261</v>
+        <v>45292</v>
       </c>
       <c r="B23" s="6">
-        <v>34.6</v>
+        <v>34.85</v>
       </c>
       <c r="C23" s="6">
+        <v>31.9</v>
+      </c>
+      <c r="D23" s="6">
         <v>34.85</v>
       </c>
-      <c r="D23" s="6">
-        <v>35.049999999999997</v>
-      </c>
       <c r="E23" s="6">
-        <v>34</v>
+        <v>31.8</v>
       </c>
       <c r="F23" s="7">
-        <v>-0.1</v>
+        <v>-2.95</v>
       </c>
       <c r="G23" s="7">
-        <v>-0.28999999999999998</v>
+        <v>-8.4600000000000009</v>
       </c>
       <c r="H23" s="8">
-        <v>95.14</v>
-      </c>
-      <c r="I23" s="9">
-        <v>8.27</v>
+        <v>72.38</v>
+      </c>
+      <c r="I23" s="7">
+        <v>-23.9</v>
       </c>
       <c r="J23" s="7">
-        <v>-24.4</v>
-      </c>
-      <c r="K23" s="16">
-        <v>1086</v>
+        <v>-1.19</v>
+      </c>
+      <c r="K23" s="8">
+        <v>72.38</v>
       </c>
       <c r="L23" s="7">
-        <v>-3.85</v>
+        <v>-1.19</v>
       </c>
       <c r="M23" s="8">
-        <v>95.14</v>
-      </c>
-      <c r="N23" s="9">
-        <v>8.27</v>
+        <v>72.38</v>
+      </c>
+      <c r="N23" s="7">
+        <v>-23.9</v>
       </c>
       <c r="O23" s="7">
-        <v>-24.4</v>
-      </c>
-      <c r="P23" s="16">
-        <v>1086</v>
+        <v>-1.19</v>
+      </c>
+      <c r="P23" s="8">
+        <v>72.38</v>
       </c>
       <c r="Q23" s="7">
-        <v>-3.85</v>
+        <v>-1.19</v>
       </c>
     </row>
     <row r="24" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="11">
-        <v>45231</v>
+        <v>45261</v>
       </c>
       <c r="B24" s="12">
-        <v>32.35</v>
+        <v>34.6</v>
       </c>
       <c r="C24" s="12">
-        <v>34.950000000000003</v>
+        <v>34.85</v>
       </c>
       <c r="D24" s="12">
-        <v>35.5</v>
+        <v>35.049999999999997</v>
       </c>
       <c r="E24" s="12">
-        <v>32</v>
-      </c>
-      <c r="F24" s="15">
-        <v>2.7</v>
-      </c>
-      <c r="G24" s="15">
-        <v>8.3699999999999992</v>
+        <v>34</v>
+      </c>
+      <c r="F24" s="13">
+        <v>-0.1</v>
+      </c>
+      <c r="G24" s="13">
+        <v>-0.28999999999999998</v>
       </c>
       <c r="H24" s="14">
-        <v>87.87</v>
-      </c>
-      <c r="I24" s="13">
-        <v>-6.24</v>
+        <v>95.14</v>
+      </c>
+      <c r="I24" s="15">
+        <v>8.27</v>
       </c>
       <c r="J24" s="13">
-        <v>-9.17</v>
-      </c>
-      <c r="K24" s="14">
-        <v>991</v>
+        <v>-24.4</v>
+      </c>
+      <c r="K24" s="16">
+        <v>1086</v>
       </c>
       <c r="L24" s="13">
-        <v>-1.27</v>
+        <v>-3.85</v>
       </c>
       <c r="M24" s="14">
-        <v>87.87</v>
-      </c>
-      <c r="N24" s="13">
-        <v>-6.24</v>
+        <v>95.14</v>
+      </c>
+      <c r="N24" s="15">
+        <v>8.27</v>
       </c>
       <c r="O24" s="13">
-        <v>-9.17</v>
-      </c>
-      <c r="P24" s="14">
-        <v>991</v>
+        <v>-24.4</v>
+      </c>
+      <c r="P24" s="16">
+        <v>1086</v>
       </c>
       <c r="Q24" s="13">
-        <v>-1.27</v>
+        <v>-3.85</v>
       </c>
     </row>
     <row r="25" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
-        <v>45200</v>
+        <v>45231</v>
       </c>
       <c r="B25" s="6">
-        <v>33.299999999999997</v>
+        <v>32.35</v>
       </c>
       <c r="C25" s="6">
-        <v>32.25</v>
+        <v>34.950000000000003</v>
       </c>
       <c r="D25" s="6">
-        <v>34.15</v>
+        <v>35.5</v>
       </c>
       <c r="E25" s="6">
-        <v>31.35</v>
-      </c>
-      <c r="F25" s="7">
-        <v>-1</v>
-      </c>
-      <c r="G25" s="7">
-        <v>-3.01</v>
+        <v>32</v>
+      </c>
+      <c r="F25" s="9">
+        <v>2.7</v>
+      </c>
+      <c r="G25" s="9">
+        <v>8.3699999999999992</v>
       </c>
       <c r="H25" s="8">
-        <v>93.72</v>
-      </c>
-      <c r="I25" s="9">
-        <v>7.28</v>
+        <v>87.87</v>
+      </c>
+      <c r="I25" s="7">
+        <v>-6.24</v>
       </c>
       <c r="J25" s="7">
-        <v>-17.600000000000001</v>
+        <v>-9.17</v>
       </c>
       <c r="K25" s="8">
-        <v>903.1</v>
+        <v>991</v>
       </c>
       <c r="L25" s="7">
-        <v>-0.43</v>
+        <v>-1.27</v>
       </c>
       <c r="M25" s="8">
-        <v>93.72</v>
-      </c>
-      <c r="N25" s="9">
-        <v>7.28</v>
+        <v>87.87</v>
+      </c>
+      <c r="N25" s="7">
+        <v>-6.24</v>
       </c>
       <c r="O25" s="7">
-        <v>-17.600000000000001</v>
+        <v>-9.17</v>
       </c>
       <c r="P25" s="8">
-        <v>903.1</v>
+        <v>991</v>
       </c>
       <c r="Q25" s="7">
-        <v>-0.43</v>
+        <v>-1.27</v>
       </c>
     </row>
     <row r="26" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="11">
-        <v>45170</v>
+        <v>45200</v>
       </c>
       <c r="B26" s="12">
-        <v>35.1</v>
+        <v>33.299999999999997</v>
       </c>
       <c r="C26" s="12">
-        <v>33.25</v>
+        <v>32.25</v>
       </c>
       <c r="D26" s="12">
-        <v>35.5</v>
+        <v>34.15</v>
       </c>
       <c r="E26" s="12">
-        <v>32.9</v>
+        <v>31.35</v>
       </c>
       <c r="F26" s="13">
-        <v>-1.7</v>
+        <v>-1</v>
       </c>
       <c r="G26" s="13">
-        <v>-4.8600000000000003</v>
+        <v>-3.01</v>
       </c>
       <c r="H26" s="14">
-        <v>87.35</v>
-      </c>
-      <c r="I26" s="13">
-        <v>-6.86</v>
+        <v>93.72</v>
+      </c>
+      <c r="I26" s="15">
+        <v>7.28</v>
       </c>
       <c r="J26" s="13">
-        <v>-16</v>
+        <v>-17.600000000000001</v>
       </c>
       <c r="K26" s="14">
-        <v>809.4</v>
-      </c>
-      <c r="L26" s="15">
-        <v>2.0099999999999998</v>
+        <v>903.1</v>
+      </c>
+      <c r="L26" s="13">
+        <v>-0.43</v>
       </c>
       <c r="M26" s="14">
-        <v>87.35</v>
-      </c>
-      <c r="N26" s="13">
-        <v>-6.86</v>
+        <v>93.72</v>
+      </c>
+      <c r="N26" s="15">
+        <v>7.28</v>
       </c>
       <c r="O26" s="13">
-        <v>-16</v>
+        <v>-17.600000000000001</v>
       </c>
       <c r="P26" s="14">
-        <v>809.4</v>
-      </c>
-      <c r="Q26" s="15">
-        <v>2.0099999999999998</v>
+        <v>903.1</v>
+      </c>
+      <c r="Q26" s="13">
+        <v>-0.43</v>
       </c>
     </row>
     <row r="27" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
-        <v>45139</v>
+        <v>45170</v>
       </c>
       <c r="B27" s="6">
-        <v>37.35</v>
+        <v>35.1</v>
       </c>
       <c r="C27" s="6">
-        <v>34.950000000000003</v>
+        <v>33.25</v>
       </c>
       <c r="D27" s="6">
-        <v>37.799999999999997</v>
+        <v>35.5</v>
       </c>
       <c r="E27" s="6">
-        <v>34.950000000000003</v>
+        <v>32.9</v>
       </c>
       <c r="F27" s="7">
-        <v>-2.35</v>
+        <v>-1.7</v>
       </c>
       <c r="G27" s="7">
-        <v>-6.3</v>
+        <v>-4.8600000000000003</v>
       </c>
       <c r="H27" s="8">
-        <v>93.79</v>
-      </c>
-      <c r="I27" s="9">
-        <v>4.75</v>
+        <v>87.35</v>
+      </c>
+      <c r="I27" s="7">
+        <v>-6.86</v>
       </c>
       <c r="J27" s="7">
-        <v>-12.2</v>
+        <v>-16</v>
       </c>
       <c r="K27" s="8">
-        <v>722.1</v>
+        <v>809.4</v>
       </c>
       <c r="L27" s="9">
-        <v>4.74</v>
+        <v>2.0099999999999998</v>
       </c>
       <c r="M27" s="8">
-        <v>93.79</v>
-      </c>
-      <c r="N27" s="9">
-        <v>4.75</v>
+        <v>87.35</v>
+      </c>
+      <c r="N27" s="7">
+        <v>-6.86</v>
       </c>
       <c r="O27" s="7">
-        <v>-12.2</v>
+        <v>-16</v>
       </c>
       <c r="P27" s="8">
-        <v>722.1</v>
+        <v>809.4</v>
       </c>
       <c r="Q27" s="9">
-        <v>4.74</v>
+        <v>2.0099999999999998</v>
       </c>
     </row>
     <row r="28" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="11">
-        <v>45108</v>
+        <v>45139</v>
       </c>
       <c r="B28" s="12">
-        <v>38.200000000000003</v>
+        <v>37.35</v>
       </c>
       <c r="C28" s="12">
-        <v>37.299999999999997</v>
+        <v>34.950000000000003</v>
       </c>
       <c r="D28" s="12">
-        <v>38.299999999999997</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="E28" s="12">
-        <v>36</v>
+        <v>34.950000000000003</v>
       </c>
       <c r="F28" s="13">
-        <v>-0.75</v>
+        <v>-2.35</v>
       </c>
       <c r="G28" s="13">
-        <v>-1.97</v>
+        <v>-6.3</v>
       </c>
       <c r="H28" s="14">
-        <v>89.53</v>
+        <v>93.79</v>
       </c>
       <c r="I28" s="15">
-        <v>1.55</v>
+        <v>4.75</v>
       </c>
       <c r="J28" s="13">
-        <v>-11.4</v>
+        <v>-12.2</v>
       </c>
       <c r="K28" s="14">
-        <v>628.29999999999995</v>
+        <v>722.1</v>
       </c>
       <c r="L28" s="15">
-        <v>7.86</v>
+        <v>4.74</v>
       </c>
       <c r="M28" s="14">
-        <v>89.53</v>
+        <v>93.79</v>
       </c>
       <c r="N28" s="15">
-        <v>1.55</v>
+        <v>4.75</v>
       </c>
       <c r="O28" s="13">
-        <v>-11.4</v>
+        <v>-12.2</v>
       </c>
       <c r="P28" s="14">
-        <v>628.29999999999995</v>
+        <v>722.1</v>
       </c>
       <c r="Q28" s="15">
-        <v>7.86</v>
+        <v>4.74</v>
       </c>
     </row>
     <row r="29" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
-        <v>45078</v>
+        <v>45108</v>
       </c>
       <c r="B29" s="6">
-        <v>38.049999999999997</v>
+        <v>38.200000000000003</v>
       </c>
       <c r="C29" s="6">
-        <v>38.049999999999997</v>
+        <v>37.299999999999997</v>
       </c>
       <c r="D29" s="6">
-        <v>39.25</v>
+        <v>38.299999999999997</v>
       </c>
       <c r="E29" s="6">
-        <v>37.75</v>
-      </c>
-      <c r="F29" s="9">
-        <v>0.15</v>
-      </c>
-      <c r="G29" s="9">
-        <v>0.4</v>
+        <v>36</v>
+      </c>
+      <c r="F29" s="7">
+        <v>-0.75</v>
+      </c>
+      <c r="G29" s="7">
+        <v>-1.97</v>
       </c>
       <c r="H29" s="8">
-        <v>88.16</v>
-      </c>
-      <c r="I29" s="7">
-        <v>-8.1199999999999992</v>
+        <v>89.53</v>
+      </c>
+      <c r="I29" s="9">
+        <v>1.55</v>
       </c>
       <c r="J29" s="7">
-        <v>-3.6</v>
+        <v>-11.4</v>
       </c>
       <c r="K29" s="8">
-        <v>538.70000000000005</v>
+        <v>628.29999999999995</v>
       </c>
       <c r="L29" s="9">
-        <v>11.9</v>
+        <v>7.86</v>
       </c>
       <c r="M29" s="8">
-        <v>88.16</v>
-      </c>
-      <c r="N29" s="7">
-        <v>-8.1199999999999992</v>
+        <v>89.53</v>
+      </c>
+      <c r="N29" s="9">
+        <v>1.55</v>
       </c>
       <c r="O29" s="7">
-        <v>-3.6</v>
+        <v>-11.4</v>
       </c>
       <c r="P29" s="8">
-        <v>538.70000000000005</v>
+        <v>628.29999999999995</v>
       </c>
       <c r="Q29" s="9">
-        <v>11.9</v>
+        <v>7.86</v>
       </c>
     </row>
     <row r="30" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="11">
-        <v>45047</v>
+        <v>45078</v>
       </c>
       <c r="B30" s="12">
-        <v>39</v>
+        <v>38.049999999999997</v>
       </c>
       <c r="C30" s="12">
-        <v>37.9</v>
+        <v>38.049999999999997</v>
       </c>
       <c r="D30" s="12">
-        <v>40.25</v>
+        <v>39.25</v>
       </c>
       <c r="E30" s="12">
-        <v>37.15</v>
-      </c>
-      <c r="F30" s="13">
-        <v>-0.8</v>
-      </c>
-      <c r="G30" s="13">
-        <v>-2.0699999999999998</v>
+        <v>37.75</v>
+      </c>
+      <c r="F30" s="15">
+        <v>0.15</v>
+      </c>
+      <c r="G30" s="15">
+        <v>0.4</v>
       </c>
       <c r="H30" s="14">
-        <v>95.96</v>
-      </c>
-      <c r="I30" s="15">
-        <v>5.45</v>
-      </c>
-      <c r="J30" s="15">
-        <v>24.1</v>
+        <v>88.16</v>
+      </c>
+      <c r="I30" s="13">
+        <v>-8.1199999999999992</v>
+      </c>
+      <c r="J30" s="13">
+        <v>-3.6</v>
       </c>
       <c r="K30" s="14">
-        <v>450.6</v>
+        <v>538.70000000000005</v>
       </c>
       <c r="L30" s="15">
-        <v>15.5</v>
+        <v>11.9</v>
       </c>
       <c r="M30" s="14">
-        <v>95.96</v>
-      </c>
-      <c r="N30" s="15">
-        <v>5.45</v>
-      </c>
-      <c r="O30" s="15">
-        <v>24.1</v>
+        <v>88.16</v>
+      </c>
+      <c r="N30" s="13">
+        <v>-8.1199999999999992</v>
+      </c>
+      <c r="O30" s="13">
+        <v>-3.6</v>
       </c>
       <c r="P30" s="14">
-        <v>450.6</v>
+        <v>538.70000000000005</v>
       </c>
       <c r="Q30" s="15">
-        <v>15.5</v>
+        <v>11.9</v>
       </c>
     </row>
     <row r="31" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
-        <v>45017</v>
+        <v>45047</v>
       </c>
       <c r="B31" s="6">
-        <v>36.65</v>
+        <v>39</v>
       </c>
       <c r="C31" s="6">
-        <v>38.700000000000003</v>
+        <v>37.9</v>
       </c>
       <c r="D31" s="6">
-        <v>39.799999999999997</v>
+        <v>40.25</v>
       </c>
       <c r="E31" s="6">
-        <v>36.200000000000003</v>
-      </c>
-      <c r="F31" s="9">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="G31" s="9">
-        <v>6.32</v>
+        <v>37.15</v>
+      </c>
+      <c r="F31" s="7">
+        <v>-0.8</v>
+      </c>
+      <c r="G31" s="7">
+        <v>-2.0699999999999998</v>
       </c>
       <c r="H31" s="8">
-        <v>91</v>
-      </c>
-      <c r="I31" s="7">
-        <v>-22.4</v>
+        <v>95.96</v>
+      </c>
+      <c r="I31" s="9">
+        <v>5.45</v>
       </c>
       <c r="J31" s="9">
-        <v>9.3800000000000008</v>
+        <v>24.1</v>
       </c>
       <c r="K31" s="8">
-        <v>354.6</v>
+        <v>450.6</v>
       </c>
       <c r="L31" s="9">
-        <v>13.4</v>
+        <v>15.5</v>
       </c>
       <c r="M31" s="8">
-        <v>91</v>
-      </c>
-      <c r="N31" s="7">
-        <v>-22.4</v>
+        <v>95.96</v>
+      </c>
+      <c r="N31" s="9">
+        <v>5.45</v>
       </c>
       <c r="O31" s="9">
-        <v>9.3800000000000008</v>
+        <v>24.1</v>
       </c>
       <c r="P31" s="8">
-        <v>354.6</v>
+        <v>450.6</v>
       </c>
       <c r="Q31" s="9">
-        <v>13.4</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="32" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="11">
-        <v>44986</v>
+        <v>45017</v>
       </c>
       <c r="B32" s="12">
-        <v>38.85</v>
+        <v>36.65</v>
       </c>
       <c r="C32" s="12">
-        <v>36.4</v>
+        <v>38.700000000000003</v>
       </c>
       <c r="D32" s="12">
-        <v>38.85</v>
+        <v>39.799999999999997</v>
       </c>
       <c r="E32" s="12">
-        <v>36.049999999999997</v>
-      </c>
-      <c r="F32" s="13">
-        <v>-2.75</v>
-      </c>
-      <c r="G32" s="13">
-        <v>-7.02</v>
+        <v>36.200000000000003</v>
+      </c>
+      <c r="F32" s="15">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="G32" s="15">
+        <v>6.32</v>
       </c>
       <c r="H32" s="14">
-        <v>117.3</v>
-      </c>
-      <c r="I32" s="15">
-        <v>60.6</v>
+        <v>91</v>
+      </c>
+      <c r="I32" s="13">
+        <v>-22.4</v>
       </c>
       <c r="J32" s="15">
-        <v>17.600000000000001</v>
+        <v>9.3800000000000008</v>
       </c>
       <c r="K32" s="14">
-        <v>263.60000000000002</v>
+        <v>354.6</v>
       </c>
       <c r="L32" s="15">
-        <v>14.9</v>
+        <v>13.4</v>
       </c>
       <c r="M32" s="14">
-        <v>117.3</v>
-      </c>
-      <c r="N32" s="15">
-        <v>60.6</v>
+        <v>91</v>
+      </c>
+      <c r="N32" s="13">
+        <v>-22.4</v>
       </c>
       <c r="O32" s="15">
-        <v>17.600000000000001</v>
+        <v>9.3800000000000008</v>
       </c>
       <c r="P32" s="14">
-        <v>263.60000000000002</v>
+        <v>354.6</v>
       </c>
       <c r="Q32" s="15">
-        <v>14.9</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="33" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5">
-        <v>44958</v>
+        <v>44986</v>
       </c>
       <c r="B33" s="6">
-        <v>36.450000000000003</v>
+        <v>38.85</v>
       </c>
       <c r="C33" s="6">
-        <v>39.15</v>
+        <v>36.4</v>
       </c>
       <c r="D33" s="6">
-        <v>39.700000000000003</v>
+        <v>38.85</v>
       </c>
       <c r="E33" s="6">
-        <v>36</v>
-      </c>
-      <c r="F33" s="9">
-        <v>2.9</v>
-      </c>
-      <c r="G33" s="9">
-        <v>8</v>
+        <v>36.049999999999997</v>
+      </c>
+      <c r="F33" s="7">
+        <v>-2.75</v>
+      </c>
+      <c r="G33" s="7">
+        <v>-7.02</v>
       </c>
       <c r="H33" s="8">
-        <v>73.06</v>
-      </c>
-      <c r="I33" s="7">
-        <v>-0.26</v>
+        <v>117.3</v>
+      </c>
+      <c r="I33" s="9">
+        <v>60.6</v>
       </c>
       <c r="J33" s="9">
-        <v>33.9</v>
+        <v>17.600000000000001</v>
       </c>
       <c r="K33" s="8">
-        <v>146.30000000000001</v>
+        <v>263.60000000000002</v>
       </c>
       <c r="L33" s="9">
-        <v>12.8</v>
+        <v>14.9</v>
       </c>
       <c r="M33" s="8">
-        <v>73.06</v>
-      </c>
-      <c r="N33" s="7">
-        <v>-0.26</v>
+        <v>117.3</v>
+      </c>
+      <c r="N33" s="9">
+        <v>60.6</v>
       </c>
       <c r="O33" s="9">
-        <v>33.9</v>
+        <v>17.600000000000001</v>
       </c>
       <c r="P33" s="8">
-        <v>146.30000000000001</v>
+        <v>263.60000000000002</v>
       </c>
       <c r="Q33" s="9">
-        <v>12.8</v>
+        <v>14.9</v>
       </c>
     </row>
     <row r="34" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="11">
-        <v>44927</v>
+        <v>44958</v>
       </c>
       <c r="B34" s="12">
-        <v>33.6</v>
+        <v>36.450000000000003</v>
       </c>
       <c r="C34" s="12">
-        <v>36.25</v>
+        <v>39.15</v>
       </c>
       <c r="D34" s="12">
-        <v>37.25</v>
+        <v>39.700000000000003</v>
       </c>
       <c r="E34" s="12">
-        <v>33.299999999999997</v>
+        <v>36</v>
       </c>
       <c r="F34" s="15">
-        <v>2.6</v>
+        <v>2.9</v>
       </c>
       <c r="G34" s="15">
-        <v>7.73</v>
+        <v>8</v>
       </c>
       <c r="H34" s="14">
-        <v>73.25</v>
+        <v>73.06</v>
       </c>
       <c r="I34" s="13">
-        <v>-41.8</v>
-      </c>
-      <c r="J34" s="13">
-        <v>-2.56</v>
+        <v>-0.26</v>
+      </c>
+      <c r="J34" s="15">
+        <v>33.9</v>
       </c>
       <c r="K34" s="14">
-        <v>73.25</v>
-      </c>
-      <c r="L34" s="13">
-        <v>-2.56</v>
+        <v>146.30000000000001</v>
+      </c>
+      <c r="L34" s="15">
+        <v>12.8</v>
       </c>
       <c r="M34" s="14">
-        <v>73.25</v>
+        <v>73.06</v>
       </c>
       <c r="N34" s="13">
-        <v>-41.8</v>
-      </c>
-      <c r="O34" s="13">
-        <v>-2.56</v>
+        <v>-0.26</v>
+      </c>
+      <c r="O34" s="15">
+        <v>33.9</v>
       </c>
       <c r="P34" s="14">
-        <v>73.25</v>
-      </c>
-      <c r="Q34" s="13">
-        <v>-2.56</v>
+        <v>146.30000000000001</v>
+      </c>
+      <c r="Q34" s="15">
+        <v>12.8</v>
       </c>
     </row>
     <row r="35" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5">
-        <v>44896</v>
+        <v>44927</v>
       </c>
       <c r="B35" s="6">
-        <v>34.4</v>
+        <v>33.6</v>
       </c>
       <c r="C35" s="6">
-        <v>33.65</v>
+        <v>36.25</v>
       </c>
       <c r="D35" s="6">
-        <v>34.799999999999997</v>
+        <v>37.25</v>
       </c>
       <c r="E35" s="6">
-        <v>33</v>
-      </c>
-      <c r="F35" s="7">
-        <v>-0.25</v>
-      </c>
-      <c r="G35" s="7">
-        <v>-0.74</v>
+        <v>33.299999999999997</v>
+      </c>
+      <c r="F35" s="9">
+        <v>2.6</v>
+      </c>
+      <c r="G35" s="9">
+        <v>7.73</v>
       </c>
       <c r="H35" s="8">
-        <v>125.8</v>
-      </c>
-      <c r="I35" s="9">
-        <v>30.1</v>
-      </c>
-      <c r="J35" s="9">
-        <v>16.3</v>
-      </c>
-      <c r="K35" s="16">
-        <v>1130</v>
-      </c>
-      <c r="L35" s="9">
-        <v>5.53</v>
+        <v>73.25</v>
+      </c>
+      <c r="I35" s="7">
+        <v>-41.8</v>
+      </c>
+      <c r="J35" s="7">
+        <v>-2.56</v>
+      </c>
+      <c r="K35" s="8">
+        <v>73.25</v>
+      </c>
+      <c r="L35" s="7">
+        <v>-2.56</v>
       </c>
       <c r="M35" s="8">
-        <v>125.8</v>
-      </c>
-      <c r="N35" s="9">
-        <v>30.1</v>
-      </c>
-      <c r="O35" s="9">
-        <v>16.3</v>
-      </c>
-      <c r="P35" s="16">
-        <v>1130</v>
-      </c>
-      <c r="Q35" s="9">
-        <v>5.53</v>
+        <v>73.25</v>
+      </c>
+      <c r="N35" s="7">
+        <v>-41.8</v>
+      </c>
+      <c r="O35" s="7">
+        <v>-2.56</v>
+      </c>
+      <c r="P35" s="8">
+        <v>73.25</v>
+      </c>
+      <c r="Q35" s="7">
+        <v>-2.56</v>
       </c>
     </row>
     <row r="36" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>44866</v>
+        <v>44896</v>
       </c>
       <c r="B36" s="12">
-        <v>30.25</v>
+        <v>34.4</v>
       </c>
       <c r="C36" s="12">
-        <v>33.9</v>
+        <v>33.65</v>
       </c>
       <c r="D36" s="12">
-        <v>34.700000000000003</v>
+        <v>34.799999999999997</v>
       </c>
       <c r="E36" s="12">
+        <v>33</v>
+      </c>
+      <c r="F36" s="13">
+        <v>-0.25</v>
+      </c>
+      <c r="G36" s="13">
+        <v>-0.74</v>
+      </c>
+      <c r="H36" s="14">
+        <v>125.8</v>
+      </c>
+      <c r="I36" s="15">
         <v>30.1</v>
       </c>
-      <c r="F36" s="15">
-        <v>3.65</v>
-      </c>
-      <c r="G36" s="15">
-        <v>12.07</v>
-      </c>
-      <c r="H36" s="14">
-        <v>96.75</v>
-      </c>
-      <c r="I36" s="13">
-        <v>-14.9</v>
-      </c>
-      <c r="J36" s="13">
-        <v>-0.8</v>
-      </c>
-      <c r="K36" s="17">
-        <v>1004</v>
+      <c r="J36" s="15">
+        <v>16.3</v>
+      </c>
+      <c r="K36" s="16">
+        <v>1130</v>
       </c>
       <c r="L36" s="15">
-        <v>4.32</v>
+        <v>5.53</v>
       </c>
       <c r="M36" s="14">
-        <v>96.75</v>
-      </c>
-      <c r="N36" s="13">
-        <v>-14.9</v>
-      </c>
-      <c r="O36" s="13">
-        <v>-0.8</v>
-      </c>
-      <c r="P36" s="17">
-        <v>1004</v>
+        <v>125.8</v>
+      </c>
+      <c r="N36" s="15">
+        <v>30.1</v>
+      </c>
+      <c r="O36" s="15">
+        <v>16.3</v>
+      </c>
+      <c r="P36" s="16">
+        <v>1130</v>
       </c>
       <c r="Q36" s="15">
-        <v>4.32</v>
+        <v>5.53</v>
       </c>
     </row>
     <row r="37" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="5">
-        <v>44835</v>
+        <v>44866</v>
       </c>
       <c r="B37" s="6">
-        <v>33.65</v>
+        <v>30.25</v>
       </c>
       <c r="C37" s="6">
-        <v>30.25</v>
+        <v>33.9</v>
       </c>
       <c r="D37" s="6">
-        <v>34.5</v>
+        <v>34.700000000000003</v>
       </c>
       <c r="E37" s="6">
-        <v>29.8</v>
-      </c>
-      <c r="F37" s="7">
-        <v>-3.55</v>
-      </c>
-      <c r="G37" s="7">
-        <v>-10.5</v>
+        <v>30.1</v>
+      </c>
+      <c r="F37" s="9">
+        <v>3.65</v>
+      </c>
+      <c r="G37" s="9">
+        <v>12.07</v>
       </c>
       <c r="H37" s="8">
-        <v>113.7</v>
-      </c>
-      <c r="I37" s="9">
-        <v>9.25</v>
-      </c>
-      <c r="J37" s="9">
-        <v>18.8</v>
-      </c>
-      <c r="K37" s="8">
-        <v>907.1</v>
+        <v>96.75</v>
+      </c>
+      <c r="I37" s="7">
+        <v>-14.9</v>
+      </c>
+      <c r="J37" s="7">
+        <v>-0.8</v>
+      </c>
+      <c r="K37" s="17">
+        <v>1004</v>
       </c>
       <c r="L37" s="9">
-        <v>4.9000000000000004</v>
+        <v>4.32</v>
       </c>
       <c r="M37" s="8">
-        <v>113.7</v>
-      </c>
-      <c r="N37" s="9">
-        <v>9.25</v>
-      </c>
-      <c r="O37" s="9">
-        <v>18.8</v>
-      </c>
-      <c r="P37" s="8">
-        <v>907.1</v>
+        <v>96.75</v>
+      </c>
+      <c r="N37" s="7">
+        <v>-14.9</v>
+      </c>
+      <c r="O37" s="7">
+        <v>-0.8</v>
+      </c>
+      <c r="P37" s="17">
+        <v>1004</v>
       </c>
       <c r="Q37" s="9">
-        <v>4.9000000000000004</v>
+        <v>4.32</v>
       </c>
     </row>
     <row r="38" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>44805</v>
+        <v>44835</v>
       </c>
       <c r="B38" s="12">
-        <v>39.1</v>
+        <v>33.65</v>
       </c>
       <c r="C38" s="12">
-        <v>33.799999999999997</v>
+        <v>30.25</v>
       </c>
       <c r="D38" s="12">
-        <v>40</v>
+        <v>34.5</v>
       </c>
       <c r="E38" s="12">
-        <v>33.6</v>
+        <v>29.8</v>
       </c>
       <c r="F38" s="13">
-        <v>-5.5</v>
+        <v>-3.55</v>
       </c>
       <c r="G38" s="13">
-        <v>-13.99</v>
+        <v>-10.5</v>
       </c>
       <c r="H38" s="14">
-        <v>104</v>
-      </c>
-      <c r="I38" s="13">
-        <v>-2.66</v>
+        <v>113.7</v>
+      </c>
+      <c r="I38" s="15">
+        <v>9.25</v>
       </c>
       <c r="J38" s="15">
-        <v>8.4</v>
+        <v>18.8</v>
       </c>
       <c r="K38" s="14">
-        <v>793.4</v>
+        <v>907.1</v>
       </c>
       <c r="L38" s="15">
-        <v>3.16</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="M38" s="14">
-        <v>104</v>
-      </c>
-      <c r="N38" s="13">
-        <v>-2.66</v>
+        <v>113.7</v>
+      </c>
+      <c r="N38" s="15">
+        <v>9.25</v>
       </c>
       <c r="O38" s="15">
-        <v>8.4</v>
+        <v>18.8</v>
       </c>
       <c r="P38" s="14">
-        <v>793.4</v>
+        <v>907.1</v>
       </c>
       <c r="Q38" s="15">
-        <v>3.16</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="39" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5">
-        <v>44774</v>
+        <v>44805</v>
       </c>
       <c r="B39" s="6">
-        <v>39</v>
+        <v>39.1</v>
       </c>
       <c r="C39" s="6">
-        <v>39.299999999999997</v>
+        <v>33.799999999999997</v>
       </c>
       <c r="D39" s="6">
         <v>40</v>
       </c>
       <c r="E39" s="6">
-        <v>38.200000000000003</v>
-      </c>
-      <c r="F39" s="9">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="G39" s="9">
-        <v>1.42</v>
+        <v>33.6</v>
+      </c>
+      <c r="F39" s="7">
+        <v>-5.5</v>
+      </c>
+      <c r="G39" s="7">
+        <v>-13.99</v>
       </c>
       <c r="H39" s="8">
-        <v>106.9</v>
-      </c>
-      <c r="I39" s="9">
-        <v>5.81</v>
+        <v>104</v>
+      </c>
+      <c r="I39" s="7">
+        <v>-2.66</v>
       </c>
       <c r="J39" s="9">
-        <v>19.2</v>
+        <v>8.4</v>
       </c>
       <c r="K39" s="8">
-        <v>689.4</v>
+        <v>793.4</v>
       </c>
       <c r="L39" s="9">
-        <v>2.42</v>
+        <v>3.16</v>
       </c>
       <c r="M39" s="8">
-        <v>106.9</v>
-      </c>
-      <c r="N39" s="9">
-        <v>5.81</v>
+        <v>104</v>
+      </c>
+      <c r="N39" s="7">
+        <v>-2.66</v>
       </c>
       <c r="O39" s="9">
-        <v>19.2</v>
+        <v>8.4</v>
       </c>
       <c r="P39" s="8">
-        <v>689.4</v>
+        <v>793.4</v>
       </c>
       <c r="Q39" s="9">
-        <v>2.42</v>
+        <v>3.16</v>
       </c>
     </row>
     <row r="40" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="11">
-        <v>44743</v>
+        <v>44774</v>
       </c>
       <c r="B40" s="12">
-        <v>39.799999999999997</v>
+        <v>39</v>
       </c>
       <c r="C40" s="12">
-        <v>38.75</v>
+        <v>39.299999999999997</v>
       </c>
       <c r="D40" s="12">
-        <v>42.2</v>
+        <v>40</v>
       </c>
       <c r="E40" s="12">
-        <v>37.5</v>
-      </c>
-      <c r="F40" s="13">
-        <v>-0.75</v>
-      </c>
-      <c r="G40" s="13">
-        <v>-1.9</v>
+        <v>38.200000000000003</v>
+      </c>
+      <c r="F40" s="15">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G40" s="15">
+        <v>1.42</v>
       </c>
       <c r="H40" s="14">
-        <v>101</v>
+        <v>106.9</v>
       </c>
       <c r="I40" s="15">
-        <v>10.4</v>
+        <v>5.81</v>
       </c>
       <c r="J40" s="15">
-        <v>21.4</v>
+        <v>19.2</v>
       </c>
       <c r="K40" s="14">
-        <v>582.5</v>
-      </c>
-      <c r="L40" s="13">
-        <v>-0.16</v>
+        <v>689.4</v>
+      </c>
+      <c r="L40" s="15">
+        <v>2.42</v>
       </c>
       <c r="M40" s="14">
-        <v>101</v>
+        <v>106.9</v>
       </c>
       <c r="N40" s="15">
-        <v>10.4</v>
+        <v>5.81</v>
       </c>
       <c r="O40" s="15">
-        <v>21.4</v>
+        <v>19.2</v>
       </c>
       <c r="P40" s="14">
-        <v>582.5</v>
-      </c>
-      <c r="Q40" s="13">
-        <v>-0.16</v>
+        <v>689.4</v>
+      </c>
+      <c r="Q40" s="15">
+        <v>2.42</v>
       </c>
     </row>
     <row r="41" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="5">
-        <v>44713</v>
+        <v>44743</v>
       </c>
       <c r="B41" s="6">
-        <v>42.65</v>
+        <v>39.799999999999997</v>
       </c>
       <c r="C41" s="6">
-        <v>39.5</v>
+        <v>38.75</v>
       </c>
       <c r="D41" s="6">
-        <v>42.7</v>
+        <v>42.2</v>
       </c>
       <c r="E41" s="6">
-        <v>38.85</v>
+        <v>37.5</v>
       </c>
       <c r="F41" s="7">
-        <v>-3.1</v>
+        <v>-0.75</v>
       </c>
       <c r="G41" s="7">
-        <v>-7.28</v>
+        <v>-1.9</v>
       </c>
       <c r="H41" s="8">
-        <v>91.46</v>
+        <v>101</v>
       </c>
       <c r="I41" s="9">
-        <v>18.3</v>
+        <v>10.4</v>
       </c>
       <c r="J41" s="9">
-        <v>7.84</v>
+        <v>21.4</v>
       </c>
       <c r="K41" s="8">
-        <v>481.4</v>
+        <v>582.5</v>
       </c>
       <c r="L41" s="7">
-        <v>-3.75</v>
+        <v>-0.16</v>
       </c>
       <c r="M41" s="8">
-        <v>91.46</v>
+        <v>101</v>
       </c>
       <c r="N41" s="9">
-        <v>18.3</v>
+        <v>10.4</v>
       </c>
       <c r="O41" s="9">
-        <v>7.84</v>
+        <v>21.4</v>
       </c>
       <c r="P41" s="8">
-        <v>481.4</v>
+        <v>582.5</v>
       </c>
       <c r="Q41" s="7">
-        <v>-3.75</v>
+        <v>-0.16</v>
       </c>
     </row>
     <row r="42" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="11">
-        <v>44682</v>
+        <v>44713</v>
       </c>
       <c r="B42" s="12">
-        <v>45.9</v>
+        <v>42.65</v>
       </c>
       <c r="C42" s="12">
-        <v>42.6</v>
+        <v>39.5</v>
       </c>
       <c r="D42" s="12">
-        <v>45.9</v>
+        <v>42.7</v>
       </c>
       <c r="E42" s="12">
-        <v>40.799999999999997</v>
+        <v>38.85</v>
       </c>
       <c r="F42" s="13">
-        <v>-3.3</v>
+        <v>-3.1</v>
       </c>
       <c r="G42" s="13">
-        <v>-7.19</v>
+        <v>-7.28</v>
       </c>
       <c r="H42" s="14">
-        <v>77.34</v>
-      </c>
-      <c r="I42" s="13">
-        <v>-7.03</v>
-      </c>
-      <c r="J42" s="13">
-        <v>-21.3</v>
+        <v>91.46</v>
+      </c>
+      <c r="I42" s="15">
+        <v>18.3</v>
+      </c>
+      <c r="J42" s="15">
+        <v>7.84</v>
       </c>
       <c r="K42" s="14">
-        <v>390</v>
+        <v>481.4</v>
       </c>
       <c r="L42" s="13">
-        <v>-6.12</v>
+        <v>-3.75</v>
       </c>
       <c r="M42" s="14">
-        <v>77.34</v>
-      </c>
-      <c r="N42" s="13">
-        <v>-7.03</v>
-      </c>
-      <c r="O42" s="13">
-        <v>-21.3</v>
+        <v>91.46</v>
+      </c>
+      <c r="N42" s="15">
+        <v>18.3</v>
+      </c>
+      <c r="O42" s="15">
+        <v>7.84</v>
       </c>
       <c r="P42" s="14">
-        <v>390</v>
+        <v>481.4</v>
       </c>
       <c r="Q42" s="13">
-        <v>-6.12</v>
+        <v>-3.75</v>
       </c>
     </row>
     <row r="43" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="5">
+        <v>44682</v>
+      </c>
+      <c r="B43" s="6">
+        <v>45.9</v>
+      </c>
+      <c r="C43" s="6">
+        <v>42.6</v>
+      </c>
+      <c r="D43" s="6">
+        <v>45.9</v>
+      </c>
+      <c r="E43" s="6">
+        <v>40.799999999999997</v>
+      </c>
+      <c r="F43" s="7">
+        <v>-3.3</v>
+      </c>
+      <c r="G43" s="7">
+        <v>-7.19</v>
+      </c>
+      <c r="H43" s="8">
+        <v>77.34</v>
+      </c>
+      <c r="I43" s="7">
+        <v>-7.03</v>
+      </c>
+      <c r="J43" s="7">
+        <v>-21.3</v>
+      </c>
+      <c r="K43" s="8">
+        <v>390</v>
+      </c>
+      <c r="L43" s="7">
+        <v>-6.12</v>
+      </c>
+      <c r="M43" s="8">
+        <v>77.34</v>
+      </c>
+      <c r="N43" s="7">
+        <v>-7.03</v>
+      </c>
+      <c r="O43" s="7">
+        <v>-21.3</v>
+      </c>
+      <c r="P43" s="8">
+        <v>390</v>
+      </c>
+      <c r="Q43" s="7">
+        <v>-6.12</v>
+      </c>
+    </row>
+    <row r="44" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="11">
         <v>44652</v>
       </c>
-      <c r="B43" s="6">
+      <c r="B44" s="12">
         <v>49.7</v>
       </c>
-      <c r="C43" s="6">
+      <c r="C44" s="12">
         <v>45.9</v>
       </c>
-      <c r="D43" s="6">
+      <c r="D44" s="12">
         <v>50.2</v>
       </c>
-      <c r="E43" s="6">
+      <c r="E44" s="12">
         <v>45.5</v>
       </c>
-      <c r="F43" s="7">
+      <c r="F44" s="13">
         <v>-4</v>
       </c>
-      <c r="G43" s="7">
+      <c r="G44" s="13">
         <v>-8.02</v>
       </c>
-      <c r="H43" s="8">
+      <c r="H44" s="14">
         <v>83.19</v>
       </c>
-      <c r="I43" s="7">
+      <c r="I44" s="13">
         <v>-16.600000000000001</v>
       </c>
-      <c r="J43" s="7">
+      <c r="J44" s="13">
         <v>-14</v>
       </c>
-      <c r="K43" s="8">
+      <c r="K44" s="14">
         <v>312.60000000000002</v>
       </c>
-      <c r="L43" s="7">
+      <c r="L44" s="13">
         <v>-1.4</v>
       </c>
-      <c r="M43" s="8">
+      <c r="M44" s="14">
         <v>83.19</v>
       </c>
-      <c r="N43" s="7">
+      <c r="N44" s="13">
         <v>-16.600000000000001</v>
       </c>
-      <c r="O43" s="7">
+      <c r="O44" s="13">
         <v>-14</v>
       </c>
-      <c r="P43" s="8">
+      <c r="P44" s="14">
         <v>312.60000000000002</v>
       </c>
-      <c r="Q43" s="7">
+      <c r="Q44" s="13">
         <v>-1.4</v>
       </c>
     </row>

</xml_diff>